<commit_message>
EA3: dashboard + doc + graficos
</commit_message>
<xml_diff>
--- a/docs/Plan_Gantt_EA1_fases.xlsx
+++ b/docs/Plan_Gantt_EA1_fases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\David Sanchez\Documents\Nueva carpeta\Ingenieria\3º\Proyecto Integrador V\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\proyecto_integrado_ea1\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6350FB8F-9C09-4384-9D8D-38E7381261E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69622ECA-2A6D-44E5-9546-D52AA19A9ED0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1023,19 +1023,64 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="15" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="6" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="7" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="8" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="9" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="10" borderId="0" xfId="10" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="3" borderId="6" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="15" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="15" fillId="3" borderId="7" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="15" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="8" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="9" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="10" borderId="0" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="16" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1044,68 +1089,23 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="6" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="7" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="8" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="9" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="10" borderId="0" xfId="10" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="3" borderId="6" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="167" fontId="15" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="3" borderId="7" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="15" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="15" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="8" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="9" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="10" borderId="0" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="13">
@@ -1721,7 +1721,7 @@
   <sheetData>
     <row r="1" spans="1:67" ht="90" customHeight="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A1" s="85"/>
-      <c r="B1" s="115" t="s">
+      <c r="B1" s="99" t="s">
         <v>62</v>
       </c>
       <c r="C1" s="83"/>
@@ -1732,28 +1732,28 @@
       <c r="H1" s="13"/>
       <c r="I1" s="13"/>
       <c r="K1" s="1"/>
-      <c r="L1" s="100" t="s">
+      <c r="L1" s="109" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="101"/>
-      <c r="N1" s="101"/>
-      <c r="O1" s="101"/>
-      <c r="P1" s="101"/>
-      <c r="Q1" s="101"/>
-      <c r="R1" s="101"/>
+      <c r="M1" s="110"/>
+      <c r="N1" s="110"/>
+      <c r="O1" s="110"/>
+      <c r="P1" s="110"/>
+      <c r="Q1" s="110"/>
+      <c r="R1" s="110"/>
       <c r="S1" s="16"/>
-      <c r="T1" s="93">
+      <c r="T1" s="108">
         <v>45964</v>
       </c>
-      <c r="U1" s="92"/>
-      <c r="V1" s="92"/>
-      <c r="W1" s="92"/>
-      <c r="X1" s="92"/>
-      <c r="Y1" s="92"/>
-      <c r="Z1" s="92"/>
-      <c r="AA1" s="92"/>
-      <c r="AB1" s="92"/>
-      <c r="AC1" s="92"/>
+      <c r="U1" s="107"/>
+      <c r="V1" s="107"/>
+      <c r="W1" s="107"/>
+      <c r="X1" s="107"/>
+      <c r="Y1" s="107"/>
+      <c r="Z1" s="107"/>
+      <c r="AA1" s="107"/>
+      <c r="AB1" s="107"/>
+      <c r="AC1" s="107"/>
     </row>
     <row r="2" spans="1:67" ht="30" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B2" s="81"/>
@@ -1766,28 +1766,28 @@
       <c r="G2" s="14"/>
       <c r="H2" s="14"/>
       <c r="I2" s="14"/>
-      <c r="L2" s="94" t="s">
+      <c r="L2" s="111" t="s">
         <v>0</v>
       </c>
-      <c r="M2" s="95"/>
-      <c r="N2" s="95"/>
-      <c r="O2" s="95"/>
-      <c r="P2" s="95"/>
-      <c r="Q2" s="95"/>
-      <c r="R2" s="95"/>
+      <c r="M2" s="112"/>
+      <c r="N2" s="112"/>
+      <c r="O2" s="112"/>
+      <c r="P2" s="112"/>
+      <c r="Q2" s="112"/>
+      <c r="R2" s="112"/>
       <c r="S2" s="16"/>
-      <c r="T2" s="91">
+      <c r="T2" s="106">
         <v>1</v>
       </c>
-      <c r="U2" s="92"/>
-      <c r="V2" s="92"/>
-      <c r="W2" s="92"/>
-      <c r="X2" s="92"/>
-      <c r="Y2" s="92"/>
-      <c r="Z2" s="92"/>
-      <c r="AA2" s="92"/>
-      <c r="AB2" s="92"/>
-      <c r="AC2" s="92"/>
+      <c r="U2" s="107"/>
+      <c r="V2" s="107"/>
+      <c r="W2" s="107"/>
+      <c r="X2" s="107"/>
+      <c r="Y2" s="107"/>
+      <c r="Z2" s="107"/>
+      <c r="AA2" s="107"/>
+      <c r="AB2" s="107"/>
+      <c r="AC2" s="107"/>
     </row>
     <row r="3" spans="1:67" s="18" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6"/>
@@ -1870,111 +1870,111 @@
       <c r="I4" s="84"/>
       <c r="J4" s="84"/>
       <c r="K4" s="84"/>
-      <c r="L4" s="88">
+      <c r="L4" s="115">
         <f>L5</f>
         <v>45964</v>
       </c>
-      <c r="M4" s="86"/>
-      <c r="N4" s="86"/>
-      <c r="O4" s="86"/>
-      <c r="P4" s="86"/>
-      <c r="Q4" s="86"/>
-      <c r="R4" s="86"/>
-      <c r="S4" s="86">
+      <c r="M4" s="113"/>
+      <c r="N4" s="113"/>
+      <c r="O4" s="113"/>
+      <c r="P4" s="113"/>
+      <c r="Q4" s="113"/>
+      <c r="R4" s="113"/>
+      <c r="S4" s="113">
         <f>S5</f>
         <v>45971</v>
       </c>
-      <c r="T4" s="86"/>
-      <c r="U4" s="86"/>
-      <c r="V4" s="86"/>
-      <c r="W4" s="86"/>
-      <c r="X4" s="86"/>
-      <c r="Y4" s="86"/>
-      <c r="Z4" s="86">
+      <c r="T4" s="113"/>
+      <c r="U4" s="113"/>
+      <c r="V4" s="113"/>
+      <c r="W4" s="113"/>
+      <c r="X4" s="113"/>
+      <c r="Y4" s="113"/>
+      <c r="Z4" s="113">
         <f>Z5</f>
         <v>45978</v>
       </c>
-      <c r="AA4" s="86"/>
-      <c r="AB4" s="86"/>
-      <c r="AC4" s="86"/>
-      <c r="AD4" s="86"/>
-      <c r="AE4" s="86"/>
-      <c r="AF4" s="86"/>
-      <c r="AG4" s="86">
+      <c r="AA4" s="113"/>
+      <c r="AB4" s="113"/>
+      <c r="AC4" s="113"/>
+      <c r="AD4" s="113"/>
+      <c r="AE4" s="113"/>
+      <c r="AF4" s="113"/>
+      <c r="AG4" s="113">
         <f>AG5</f>
         <v>45985</v>
       </c>
-      <c r="AH4" s="86"/>
-      <c r="AI4" s="86"/>
-      <c r="AJ4" s="86"/>
-      <c r="AK4" s="86"/>
-      <c r="AL4" s="86"/>
-      <c r="AM4" s="86"/>
-      <c r="AN4" s="86">
+      <c r="AH4" s="113"/>
+      <c r="AI4" s="113"/>
+      <c r="AJ4" s="113"/>
+      <c r="AK4" s="113"/>
+      <c r="AL4" s="113"/>
+      <c r="AM4" s="113"/>
+      <c r="AN4" s="113">
         <f>AN5</f>
         <v>45992</v>
       </c>
-      <c r="AO4" s="86"/>
-      <c r="AP4" s="86"/>
-      <c r="AQ4" s="86"/>
-      <c r="AR4" s="86"/>
-      <c r="AS4" s="86"/>
-      <c r="AT4" s="86"/>
-      <c r="AU4" s="86">
+      <c r="AO4" s="113"/>
+      <c r="AP4" s="113"/>
+      <c r="AQ4" s="113"/>
+      <c r="AR4" s="113"/>
+      <c r="AS4" s="113"/>
+      <c r="AT4" s="113"/>
+      <c r="AU4" s="113">
         <f>AU5</f>
         <v>45999</v>
       </c>
-      <c r="AV4" s="86"/>
-      <c r="AW4" s="86"/>
-      <c r="AX4" s="86"/>
-      <c r="AY4" s="86"/>
-      <c r="AZ4" s="86"/>
-      <c r="BA4" s="86"/>
-      <c r="BB4" s="86">
+      <c r="AV4" s="113"/>
+      <c r="AW4" s="113"/>
+      <c r="AX4" s="113"/>
+      <c r="AY4" s="113"/>
+      <c r="AZ4" s="113"/>
+      <c r="BA4" s="113"/>
+      <c r="BB4" s="113">
         <f>BB5</f>
         <v>46006</v>
       </c>
-      <c r="BC4" s="86"/>
-      <c r="BD4" s="86"/>
-      <c r="BE4" s="86"/>
-      <c r="BF4" s="86"/>
-      <c r="BG4" s="86"/>
-      <c r="BH4" s="86"/>
-      <c r="BI4" s="86">
+      <c r="BC4" s="113"/>
+      <c r="BD4" s="113"/>
+      <c r="BE4" s="113"/>
+      <c r="BF4" s="113"/>
+      <c r="BG4" s="113"/>
+      <c r="BH4" s="113"/>
+      <c r="BI4" s="113">
         <f>BI5</f>
         <v>46013</v>
       </c>
-      <c r="BJ4" s="86"/>
-      <c r="BK4" s="86"/>
-      <c r="BL4" s="86"/>
-      <c r="BM4" s="86"/>
-      <c r="BN4" s="86"/>
-      <c r="BO4" s="87"/>
+      <c r="BJ4" s="113"/>
+      <c r="BK4" s="113"/>
+      <c r="BL4" s="113"/>
+      <c r="BM4" s="113"/>
+      <c r="BN4" s="113"/>
+      <c r="BO4" s="114"/>
     </row>
     <row r="5" spans="1:67" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="96"/>
-      <c r="B5" s="97" t="s">
+      <c r="A5" s="100"/>
+      <c r="B5" s="101" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="97" t="s">
+      <c r="C5" s="101" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="99" t="s">
+      <c r="D5" s="103" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="89" t="s">
+      <c r="E5" s="105" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="89" t="s">
+      <c r="F5" s="105" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="89" t="s">
+      <c r="G5" s="105" t="s">
         <v>6</v>
       </c>
-      <c r="H5" s="89" t="s">
+      <c r="H5" s="105" t="s">
         <v>34</v>
       </c>
-      <c r="I5" s="89" t="s">
+      <c r="I5" s="105" t="s">
         <v>35</v>
       </c>
       <c r="J5" s="84"/>
@@ -2205,15 +2205,15 @@
       </c>
     </row>
     <row r="6" spans="1:67" s="18" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="96"/>
-      <c r="B6" s="98"/>
-      <c r="C6" s="98"/>
-      <c r="D6" s="90"/>
-      <c r="E6" s="90"/>
-      <c r="F6" s="90"/>
-      <c r="G6" s="90"/>
-      <c r="H6" s="90"/>
-      <c r="I6" s="90"/>
+      <c r="A6" s="100"/>
+      <c r="B6" s="102"/>
+      <c r="C6" s="102"/>
+      <c r="D6" s="104"/>
+      <c r="E6" s="104"/>
+      <c r="F6" s="104"/>
+      <c r="G6" s="104"/>
+      <c r="H6" s="104"/>
+      <c r="I6" s="104"/>
       <c r="J6" s="84"/>
       <c r="K6" s="84"/>
       <c r="L6" s="26" t="str">
@@ -2594,7 +2594,7 @@
       <c r="B9" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="102" t="s">
+      <c r="C9" s="86" t="s">
         <v>17</v>
       </c>
       <c r="D9" s="40"/>
@@ -2612,7 +2612,7 @@
       <c r="H9" s="42" t="s">
         <v>36</v>
       </c>
-      <c r="I9" s="109" t="s">
+      <c r="I9" s="93" t="s">
         <v>38</v>
       </c>
       <c r="J9" s="9"/>
@@ -2682,7 +2682,7 @@
       <c r="B10" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="103" t="s">
+      <c r="C10" s="87" t="s">
         <v>18</v>
       </c>
       <c r="D10" s="44"/>
@@ -2700,7 +2700,7 @@
       <c r="H10" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="I10" s="110" t="s">
+      <c r="I10" s="94" t="s">
         <v>39</v>
       </c>
       <c r="J10" s="9"/>
@@ -2765,12 +2765,12 @@
       <c r="BN10" s="43"/>
       <c r="BO10" s="43"/>
     </row>
-    <row r="11" spans="1:67" s="38" customFormat="1" ht="39" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:67" s="38" customFormat="1" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6"/>
       <c r="B11" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="103" t="s">
+      <c r="C11" s="87" t="s">
         <v>19</v>
       </c>
       <c r="D11" s="44"/>
@@ -2788,7 +2788,7 @@
       <c r="H11" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="I11" s="110" t="s">
+      <c r="I11" s="94" t="s">
         <v>40</v>
       </c>
       <c r="J11" s="9"/>
@@ -2871,12 +2871,12 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:67" s="38" customFormat="1" ht="39" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:67" s="38" customFormat="1" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="85"/>
       <c r="B13" s="53" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="104" t="s">
+      <c r="C13" s="88" t="s">
         <v>20</v>
       </c>
       <c r="D13" s="54"/>
@@ -2891,10 +2891,10 @@
         <f>F13+4</f>
         <v>45974</v>
       </c>
-      <c r="H13" s="111" t="s">
+      <c r="H13" s="95" t="s">
         <v>14</v>
       </c>
-      <c r="I13" s="111" t="s">
+      <c r="I13" s="95" t="s">
         <v>42</v>
       </c>
       <c r="J13" s="9"/>
@@ -2964,7 +2964,7 @@
       <c r="B14" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="104" t="s">
+      <c r="C14" s="88" t="s">
         <v>21</v>
       </c>
       <c r="D14" s="54"/>
@@ -2979,10 +2979,10 @@
         <f>F14+5</f>
         <v>45977</v>
       </c>
-      <c r="H14" s="111" t="s">
+      <c r="H14" s="95" t="s">
         <v>22</v>
       </c>
-      <c r="I14" s="111" t="s">
+      <c r="I14" s="95" t="s">
         <v>43</v>
       </c>
       <c r="J14" s="9"/>
@@ -3052,7 +3052,7 @@
       <c r="B15" s="53" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="104" t="s">
+      <c r="C15" s="88" t="s">
         <v>26</v>
       </c>
       <c r="D15" s="54"/>
@@ -3067,10 +3067,10 @@
         <f>F15+3</f>
         <v>45980</v>
       </c>
-      <c r="H15" s="111" t="s">
+      <c r="H15" s="95" t="s">
         <v>15</v>
       </c>
-      <c r="I15" s="111" t="s">
+      <c r="I15" s="95" t="s">
         <v>44</v>
       </c>
       <c r="J15" s="9"/>
@@ -3140,7 +3140,7 @@
       <c r="B16" s="53" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="105" t="s">
+      <c r="C16" s="89" t="s">
         <v>27</v>
       </c>
       <c r="D16" s="54"/>
@@ -3155,10 +3155,10 @@
         <f>F16+2</f>
         <v>45979</v>
       </c>
-      <c r="H16" s="111" t="s">
+      <c r="H16" s="95" t="s">
         <v>41</v>
       </c>
-      <c r="I16" s="104" t="s">
+      <c r="I16" s="88" t="s">
         <v>45</v>
       </c>
       <c r="J16" s="9"/>
@@ -3302,7 +3302,7 @@
       <c r="B18" s="63" t="s">
         <v>46</v>
       </c>
-      <c r="C18" s="106" t="s">
+      <c r="C18" s="90" t="s">
         <v>28</v>
       </c>
       <c r="D18" s="64"/>
@@ -3317,10 +3317,10 @@
         <f>F18+5</f>
         <v>45984</v>
       </c>
-      <c r="H18" s="112" t="s">
+      <c r="H18" s="96" t="s">
         <v>23</v>
       </c>
-      <c r="I18" s="112" t="s">
+      <c r="I18" s="96" t="s">
         <v>49</v>
       </c>
       <c r="J18" s="9"/>
@@ -3390,7 +3390,7 @@
       <c r="B19" s="63" t="s">
         <v>47</v>
       </c>
-      <c r="C19" s="106" t="s">
+      <c r="C19" s="90" t="s">
         <v>29</v>
       </c>
       <c r="D19" s="64"/>
@@ -3405,10 +3405,10 @@
         <f>F19+4</f>
         <v>45989</v>
       </c>
-      <c r="H19" s="112" t="s">
+      <c r="H19" s="96" t="s">
         <v>46</v>
       </c>
-      <c r="I19" s="112" t="s">
+      <c r="I19" s="96" t="s">
         <v>50</v>
       </c>
       <c r="J19" s="9"/>
@@ -3478,7 +3478,7 @@
       <c r="B20" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="C20" s="106" t="s">
+      <c r="C20" s="90" t="s">
         <v>30</v>
       </c>
       <c r="D20" s="64"/>
@@ -3493,10 +3493,10 @@
         <f>F20+5</f>
         <v>45995</v>
       </c>
-      <c r="H20" s="112" t="s">
+      <c r="H20" s="96" t="s">
         <v>47</v>
       </c>
-      <c r="I20" s="112" t="s">
+      <c r="I20" s="96" t="s">
         <v>51</v>
       </c>
       <c r="J20" s="9"/>
@@ -3566,7 +3566,7 @@
       <c r="B21" s="63" t="s">
         <v>57</v>
       </c>
-      <c r="C21" s="106" t="s">
+      <c r="C21" s="90" t="s">
         <v>31</v>
       </c>
       <c r="D21" s="64"/>
@@ -3581,10 +3581,10 @@
         <f>F21+4</f>
         <v>46000</v>
       </c>
-      <c r="H21" s="112" t="s">
+      <c r="H21" s="96" t="s">
         <v>48</v>
       </c>
-      <c r="I21" s="112" t="s">
+      <c r="I21" s="96" t="s">
         <v>52</v>
       </c>
       <c r="J21" s="9"/>
@@ -3728,7 +3728,7 @@
       <c r="B23" s="73" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="113" t="s">
+      <c r="C23" s="97" t="s">
         <v>53</v>
       </c>
       <c r="D23" s="74"/>
@@ -3743,10 +3743,10 @@
         <f>F23+3</f>
         <v>45984</v>
       </c>
-      <c r="H23" s="108" t="s">
+      <c r="H23" s="92" t="s">
         <v>47</v>
       </c>
-      <c r="I23" s="114" t="s">
+      <c r="I23" s="98" t="s">
         <v>59</v>
       </c>
       <c r="J23" s="9"/>
@@ -3816,7 +3816,7 @@
       <c r="B24" s="73" t="s">
         <v>55</v>
       </c>
-      <c r="C24" s="107" t="s">
+      <c r="C24" s="91" t="s">
         <v>32</v>
       </c>
       <c r="D24" s="74"/>
@@ -3831,10 +3831,10 @@
         <f>F24+4</f>
         <v>45988</v>
       </c>
-      <c r="H24" s="108" t="s">
+      <c r="H24" s="92" t="s">
         <v>54</v>
       </c>
-      <c r="I24" s="108" t="s">
+      <c r="I24" s="92" t="s">
         <v>61</v>
       </c>
       <c r="J24" s="9"/>
@@ -3904,7 +3904,7 @@
       <c r="B25" s="73" t="s">
         <v>56</v>
       </c>
-      <c r="C25" s="107" t="s">
+      <c r="C25" s="91" t="s">
         <v>33</v>
       </c>
       <c r="D25" s="74"/>
@@ -3919,10 +3919,10 @@
         <f>F25+3</f>
         <v>45992</v>
       </c>
-      <c r="H25" s="108" t="s">
+      <c r="H25" s="92" t="s">
         <v>58</v>
       </c>
-      <c r="I25" s="108" t="s">
+      <c r="I25" s="92" t="s">
         <v>60</v>
       </c>
       <c r="J25" s="9"/>
@@ -4073,19 +4073,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="T2:AC2"/>
-    <mergeCell ref="T1:AC1"/>
-    <mergeCell ref="L1:R1"/>
-    <mergeCell ref="L2:R2"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="I5:I6"/>
     <mergeCell ref="BI4:BO4"/>
     <mergeCell ref="L4:R4"/>
     <mergeCell ref="S4:Y4"/>
@@ -4094,6 +4081,19 @@
     <mergeCell ref="AN4:AT4"/>
     <mergeCell ref="AU4:BA4"/>
     <mergeCell ref="BB4:BH4"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="T2:AC2"/>
+    <mergeCell ref="T1:AC1"/>
+    <mergeCell ref="L1:R1"/>
+    <mergeCell ref="L2:R2"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="C5:C6"/>
   </mergeCells>
   <phoneticPr fontId="24" type="noConversion"/>
   <conditionalFormatting sqref="E7:E26">
@@ -4198,6 +4198,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="28" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="60f5a4f2d2b0abadcf532d48ebf9cb71">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7dd78129e6a1811f84807ad11c651531" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -4509,15 +4518,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -4539,6 +4539,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97245281-08F3-4104-84BD-39F3D8CFB195}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C2348D59-3426-404A-A0C5-6456F6613EDB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4559,14 +4567,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97245281-08F3-4104-84BD-39F3D8CFB195}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82239A0-E68C-493F-BEE6-C77FEA397FD6}">
   <ds:schemaRefs>

</xml_diff>